<commit_message>
Second and third implementations of the SA
</commit_message>
<xml_diff>
--- a/metaheuristic/result.xlsx
+++ b/metaheuristic/result.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reddr\Documents\Scandiatransplant_modelling\metaheuristic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF785579-2CEB-4F38-91CB-47E84A996FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD5AD72-1C9A-4E36-B2B2-2F5C5D416DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="25760" windowHeight="15440" activeTab="1" xr2:uid="{90D588C5-8560-46EF-A81F-A53859D19916}"/>
+    <workbookView xWindow="-21990" yWindow="3300" windowWidth="21600" windowHeight="12645" xr2:uid="{90D588C5-8560-46EF-A81F-A53859D19916}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Evaluating the plane" sheetId="3" r:id="rId2"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId3"/>
+    <sheet name="SA_V2" sheetId="4" r:id="rId1"/>
+    <sheet name="SA_V3" sheetId="5" r:id="rId2"/>
+    <sheet name="Sa V1" sheetId="1" r:id="rId3"/>
+    <sheet name="Evaluating the plane" sheetId="3" r:id="rId4"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="162">
   <si>
     <t>sa_log_2026-02-24_17-21-29</t>
   </si>
@@ -326,6 +328,204 @@
   </si>
   <si>
     <t>score</t>
+  </si>
+  <si>
+    <t>matching_20260306_120820</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_11-20-31</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_12-39-20</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_13-15-16</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_13-42-34</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_14-12-01</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_14-39-16</t>
+  </si>
+  <si>
+    <t>matching_20260306_155849</t>
+  </si>
+  <si>
+    <t>Different objective function?</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_15-06-11</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_16-03-25</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_16-37-22</t>
+  </si>
+  <si>
+    <t>matching_20260306_160958</t>
+  </si>
+  <si>
+    <t>matching_20260306_162344</t>
+  </si>
+  <si>
+    <t>matching_20260306_163118</t>
+  </si>
+  <si>
+    <t>matching_20260306_163853</t>
+  </si>
+  <si>
+    <t>matching_20260306_172055</t>
+  </si>
+  <si>
+    <t>matching_20260306_173241</t>
+  </si>
+  <si>
+    <t>matching_20260306_175456</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_17-08-19</t>
+  </si>
+  <si>
+    <t>mismatch_w</t>
+  </si>
+  <si>
+    <t>distance_w</t>
+  </si>
+  <si>
+    <t>Ratio w1 w2</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_17-56-38</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_18-40-20</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_19-08-10</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_19-38-21</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_20-40-31</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_21-09-55</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_21-38-00</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_22-06-29</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_22-34-45</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_23-03-21</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-06_23-31-52</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_00-59-07</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_01-28-05</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_01-56-14</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_02-24-20</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_02-52-49</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_03-21-00</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_03-49-27</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_04-17-30</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_04-45-42</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_05-13-45</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_05-42-04</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_06-10-39</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_06-38-38</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_07-06-36</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_07-35-04</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_08-03-01</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_08-30-53</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_08-58-57</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_09-27-05</t>
+  </si>
+  <si>
+    <t>sa_log_2026-03-07_09-55-27</t>
+  </si>
+  <si>
+    <t>matching_20260307_122637</t>
+  </si>
+  <si>
+    <t>matching_20260307_123609</t>
+  </si>
+  <si>
+    <t>matching_20260307_124555</t>
+  </si>
+  <si>
+    <t>matching_20260307_125708</t>
+  </si>
+  <si>
+    <t>matching_20260307_132215</t>
+  </si>
+  <si>
+    <t>matching_20260307_134603</t>
+  </si>
+  <si>
+    <t>matching_20260307_135442</t>
+  </si>
+  <si>
+    <t>matching_20260307_140229</t>
+  </si>
+  <si>
+    <t>matching_20260307_141025</t>
+  </si>
+  <si>
+    <t>matching_20260307_143414</t>
+  </si>
+  <si>
+    <t>matching_20260307_144239</t>
+  </si>
+  <si>
+    <t>matching_20260307_145054</t>
   </si>
 </sst>
 </file>
@@ -333,10 +533,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="166" formatCode="0.00000000000000"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.00000000000000"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -344,16 +544,44 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -361,25 +589,153 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="9">
     <dxf>
-      <numFmt numFmtId="167" formatCode="0.000000"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="165" formatCode="0.000000"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -395,19 +751,70 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1EDB3E08-0EA0-4602-9D6B-1F799E50ACBD}" name="Tabla2" displayName="Tabla2" ref="A1:J22" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6">
+  <autoFilter ref="A1:J22" xr:uid="{1EDB3E08-0EA0-4602-9D6B-1F799E50ACBD}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{7D566F81-2CA3-46AE-9AFF-E32DFD72AF7C}" name="Run"/>
+    <tableColumn id="2" xr3:uid="{654000B6-B6F3-4000-A722-192F43AEC2FF}" name="Columna1"/>
+    <tableColumn id="3" xr3:uid="{E7F87D89-B003-4138-B5EF-3F406FC01AA9}" name="best_eval"/>
+    <tableColumn id="10" xr3:uid="{5303D8CF-1F75-4585-A684-F0656BD02960}" name="mismatch_w"/>
+    <tableColumn id="4" xr3:uid="{4405B6C8-267C-4DF7-ACC1-0921D18B4766}" name="distance_w"/>
+    <tableColumn id="5" xr3:uid="{28D0A62B-89AF-4DD5-9635-9A67DD6AFEE6}" name="match log"/>
+    <tableColumn id="6" xr3:uid="{3DADEE76-810E-4E8A-91F8-DE33D4E4B2F7}" name="Average mismatch"/>
+    <tableColumn id="7" xr3:uid="{5D261115-3890-4840-B42F-6B6E29A7B719}" name="Distance"/>
+    <tableColumn id="8" xr3:uid="{B340233E-E552-4351-B6A1-3F44AA7965B0}" name="equity_score"/>
+    <tableColumn id="9" xr3:uid="{88B0E6C8-91AA-4048-8F1A-01B0EC87113D}" name="Ratio w1 w2" dataDxfId="5">
+      <calculatedColumnFormula>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DDEDD92C-6A24-4C02-A69E-EAF4A19948C1}" name="Tabla3" displayName="Tabla3" ref="A1:J22" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="3" tableBorderDxfId="2">
+  <autoFilter ref="A1:J22" xr:uid="{DDEDD92C-6A24-4C02-A69E-EAF4A19948C1}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{6D394A0D-845C-4539-92CF-7A1BFB0D49C9}" name="Run"/>
+    <tableColumn id="2" xr3:uid="{850FCB11-EC36-4509-B1AF-9C314669DBD0}" name="Columna1"/>
+    <tableColumn id="3" xr3:uid="{FA52FFFB-E24D-47EE-9FB7-4176C0680B64}" name="best_eval"/>
+    <tableColumn id="4" xr3:uid="{70FC1488-A25D-41A2-933D-9B551451D7D9}" name="mismatch_w"/>
+    <tableColumn id="5" xr3:uid="{8C6FE220-0612-4583-A1F1-2B804FD6BB69}" name="distance_w"/>
+    <tableColumn id="6" xr3:uid="{48D69A99-F392-46BF-82CA-CAD30BEAABB9}" name="match log"/>
+    <tableColumn id="7" xr3:uid="{25FEF3C0-85FB-45DC-9692-E431372801FA}" name="Average mismatch"/>
+    <tableColumn id="8" xr3:uid="{4C214194-CAC3-46D0-9A22-9B7F4A4B5A4A}" name="Distance"/>
+    <tableColumn id="9" xr3:uid="{6F6314E1-6BB1-4AEC-92EE-4FAA84E990B8}" name="equity_score"/>
+    <tableColumn id="10" xr3:uid="{4CE52B17-55BE-4F69-9652-7CABD524B489}" name="Ratio w1 w2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{86E240C2-39CF-478F-86D0-D49751792C9A}" name="Tabla1" displayName="Tabla1" ref="A1:H22" totalsRowShown="0">
-  <autoFilter ref="A1:H22" xr:uid="{86E240C2-39CF-478F-86D0-D49751792C9A}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H22">
-    <sortCondition descending="1" ref="C1:C22"/>
+  <autoFilter ref="A1:H22" xr:uid="{86E240C2-39CF-478F-86D0-D49751792C9A}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="1.755074"/>
+        <filter val="1.755095"/>
+        <filter val="1.755120"/>
+        <filter val="1.755139"/>
+        <filter val="1.755142"/>
+        <filter val="1.755147"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:H20">
+    <sortCondition descending="1" ref="H1:H22"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="8" xr3:uid="{883421A0-50AC-436D-8DF6-AD7687F04C56}" name="Run"/>
     <tableColumn id="1" xr3:uid="{69477D73-69D2-4BD1-AEFF-94E6CAD95648}" name="Columna1"/>
-    <tableColumn id="2" xr3:uid="{7DC9CF1A-E9CA-4193-AD86-A0034182B08F}" name="best_eval" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{7DC9CF1A-E9CA-4193-AD86-A0034182B08F}" name="best_eval" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{E64A8894-285D-4055-81ED-001E6DF5F8F0}" name="best_solution"/>
     <tableColumn id="4" xr3:uid="{0FC83BD2-0A7F-441E-98CE-C21D7F31CBCE}" name="match log"/>
     <tableColumn id="5" xr3:uid="{2273C947-75F3-469F-9AA6-740627EEC19C}" name="Average mismatch"/>
-    <tableColumn id="6" xr3:uid="{57F53F87-10A1-43BA-B2F8-72D1EA20F21E}" name="Distance" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{57F53F87-10A1-43BA-B2F8-72D1EA20F21E}" name="Distance" dataDxfId="0"/>
     <tableColumn id="7" xr3:uid="{C3203D00-78D9-4294-AACB-D0FF44370A14}" name="equity_score"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -730,6 +1137,1159 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BC5A0C5-DF2F-4BCE-A6E5-6A3FD8B0D90A}">
+  <dimension ref="A1:L28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="3" max="4" width="18.5703125" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" customWidth="1"/>
+    <col min="6" max="6" width="32.28515625" customWidth="1"/>
+    <col min="7" max="7" width="25.42578125" customWidth="1"/>
+    <col min="8" max="9" width="17.42578125" customWidth="1"/>
+    <col min="10" max="10" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2">
+        <v>1.4678074212280099</v>
+      </c>
+      <c r="D2">
+        <v>29.250767826673499</v>
+      </c>
+      <c r="E2">
+        <v>500.90927710559703</v>
+      </c>
+      <c r="F2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G2">
+        <v>2.0072727272727202</v>
+      </c>
+      <c r="H2">
+        <v>210025.35456030801</v>
+      </c>
+      <c r="I2">
+        <v>0.89737266182623499</v>
+      </c>
+      <c r="J2">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>5.8395340560855942E-2</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D3">
+        <v>971.196327140211</v>
+      </c>
+      <c r="E3">
+        <v>913.58427622260001</v>
+      </c>
+      <c r="F3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G3">
+        <v>1.80727272727272</v>
+      </c>
+      <c r="H3">
+        <v>303823.543776009</v>
+      </c>
+      <c r="I3">
+        <v>0.87790928015963798</v>
+      </c>
+      <c r="J3">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0630615613874395</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D4">
+        <v>391.20547966444502</v>
+      </c>
+      <c r="E4">
+        <v>376.99985576192898</v>
+      </c>
+      <c r="F4" t="s">
+        <v>108</v>
+      </c>
+      <c r="G4">
+        <v>1.79727272727272</v>
+      </c>
+      <c r="H4">
+        <v>304047.56038400601</v>
+      </c>
+      <c r="I4">
+        <v>0.88053830611493</v>
+      </c>
+      <c r="J4">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0376807144231024</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D5">
+        <v>51.1429296699297</v>
+      </c>
+      <c r="E5">
+        <v>52.004636025417099</v>
+      </c>
+      <c r="F5" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5">
+        <v>1.8081818181818099</v>
+      </c>
+      <c r="H5">
+        <v>306265.96964544302</v>
+      </c>
+      <c r="I5">
+        <v>0.85551973458411601</v>
+      </c>
+      <c r="J5">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>0.9834302012023266</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D6">
+        <v>107.19415158678299</v>
+      </c>
+      <c r="E6">
+        <v>105.855156619376</v>
+      </c>
+      <c r="F6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G6">
+        <v>1.8090909090909</v>
+      </c>
+      <c r="H6">
+        <v>318538.18377070699</v>
+      </c>
+      <c r="I6">
+        <v>0.85074955429374499</v>
+      </c>
+      <c r="J6">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0126493126095086</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D7">
+        <v>873.39857956757396</v>
+      </c>
+      <c r="E7">
+        <v>828.58469969218402</v>
+      </c>
+      <c r="F7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G7">
+        <v>1.7881818181818101</v>
+      </c>
+      <c r="H7">
+        <v>317926.70649846998</v>
+      </c>
+      <c r="I7">
+        <v>0.83472122390202197</v>
+      </c>
+      <c r="J7">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0540848508209699</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D8">
+        <v>367.069106645484</v>
+      </c>
+      <c r="E8">
+        <v>358.45450085314002</v>
+      </c>
+      <c r="F8" t="s">
+        <v>112</v>
+      </c>
+      <c r="G8">
+        <v>1.80181818181818</v>
+      </c>
+      <c r="H8">
+        <v>301302.76927731099</v>
+      </c>
+      <c r="I8">
+        <v>0.87448656459218499</v>
+      </c>
+      <c r="J8">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0240326339098569</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D9">
+        <v>314.37765776341001</v>
+      </c>
+      <c r="E9">
+        <v>302.061158650116</v>
+      </c>
+      <c r="F9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G9">
+        <v>1.8027272727272701</v>
+      </c>
+      <c r="H9">
+        <v>308467.99058907002</v>
+      </c>
+      <c r="I9">
+        <v>0.85407178497681702</v>
+      </c>
+      <c r="J9">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0407748522462648</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10">
+        <v>1.5499327684320601</v>
+      </c>
+      <c r="D10">
+        <v>84.6255989756052</v>
+      </c>
+      <c r="E10">
+        <v>265.10166302991598</v>
+      </c>
+      <c r="F10" t="s">
+        <v>114</v>
+      </c>
+      <c r="G10">
+        <v>1.88636363636363</v>
+      </c>
+      <c r="H10">
+        <v>253311.47149237699</v>
+      </c>
+      <c r="I10">
+        <v>0.90125296163750801</v>
+      </c>
+      <c r="J10">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>0.31921941948004845</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11">
+        <v>1.56878920827404</v>
+      </c>
+      <c r="D11">
+        <v>126.590912020693</v>
+      </c>
+      <c r="E11">
+        <v>18.422362550585198</v>
+      </c>
+      <c r="F11" t="s">
+        <v>150</v>
+      </c>
+      <c r="G11">
+        <v>1.7981818181818101</v>
+      </c>
+      <c r="H11">
+        <v>306016.17894535401</v>
+      </c>
+      <c r="I11">
+        <v>0.86373732573926698</v>
+      </c>
+      <c r="J11">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>6.8715894431613904</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D12">
+        <v>434.14893037516799</v>
+      </c>
+      <c r="E12">
+        <v>424.03064911580702</v>
+      </c>
+      <c r="F12" t="s">
+        <v>151</v>
+      </c>
+      <c r="G12">
+        <v>1.7936363636363599</v>
+      </c>
+      <c r="H12">
+        <v>313454.51400252199</v>
+      </c>
+      <c r="I12">
+        <v>0.89244102933400005</v>
+      </c>
+      <c r="J12">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0238621460039734</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13">
+        <v>1.56878920827404</v>
+      </c>
+      <c r="D13">
+        <v>651.85909188269602</v>
+      </c>
+      <c r="E13">
+        <v>32.287128541107698</v>
+      </c>
+      <c r="F13" t="s">
+        <v>152</v>
+      </c>
+      <c r="G13">
+        <v>1.8027272727272701</v>
+      </c>
+      <c r="H13">
+        <v>326850.50367636897</v>
+      </c>
+      <c r="I13">
+        <v>0.85842347460000001</v>
+      </c>
+      <c r="J13">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>20.189441468997607</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C14">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D14">
+        <v>420.82173827692299</v>
+      </c>
+      <c r="E14">
+        <v>420.38725991794001</v>
+      </c>
+      <c r="F14" t="s">
+        <v>153</v>
+      </c>
+      <c r="G14">
+        <v>1.8036363636363599</v>
+      </c>
+      <c r="H14">
+        <v>315216.061976047</v>
+      </c>
+      <c r="I14">
+        <v>0.83989421301021405</v>
+      </c>
+      <c r="J14">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0010335193294577</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>122</v>
+      </c>
+      <c r="C15">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D15">
+        <v>272.979674928625</v>
+      </c>
+      <c r="E15">
+        <v>272.05672288388001</v>
+      </c>
+      <c r="F15" t="s">
+        <v>154</v>
+      </c>
+      <c r="G15">
+        <v>1.7963636363636299</v>
+      </c>
+      <c r="H15">
+        <v>321487.84195337998</v>
+      </c>
+      <c r="I15">
+        <v>0.87729028227749395</v>
+      </c>
+      <c r="J15">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0033924985751552</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>123</v>
+      </c>
+      <c r="C16">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D16">
+        <v>998.40288781049503</v>
+      </c>
+      <c r="E16">
+        <v>968.760443203519</v>
+      </c>
+      <c r="F16" t="s">
+        <v>155</v>
+      </c>
+      <c r="G16">
+        <v>1.7854545454545401</v>
+      </c>
+      <c r="H16">
+        <v>315651.41191506502</v>
+      </c>
+      <c r="I16">
+        <v>0.86938589848796</v>
+      </c>
+      <c r="J16">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0305983226451254</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D17">
+        <v>289.91511570772298</v>
+      </c>
+      <c r="E17">
+        <v>280.68342604497502</v>
+      </c>
+      <c r="F17" t="s">
+        <v>156</v>
+      </c>
+      <c r="G17">
+        <v>1.79454545454545</v>
+      </c>
+      <c r="H17">
+        <v>320945.45234076801</v>
+      </c>
+      <c r="I17">
+        <v>0.82881469012791797</v>
+      </c>
+      <c r="J17">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0328900419694489</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18">
+        <v>1.55352823382093</v>
+      </c>
+      <c r="D18">
+        <v>155.47842110760001</v>
+      </c>
+      <c r="E18">
+        <v>394.002153462102</v>
+      </c>
+      <c r="F18" t="s">
+        <v>157</v>
+      </c>
+      <c r="G18">
+        <v>1.88090909090909</v>
+      </c>
+      <c r="H18">
+        <v>252672.75854614499</v>
+      </c>
+      <c r="I18">
+        <v>0.92192334529723996</v>
+      </c>
+      <c r="J18">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>0.39461312518576136</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C19">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D19">
+        <v>172.37587204099199</v>
+      </c>
+      <c r="E19">
+        <v>162.53229285647299</v>
+      </c>
+      <c r="F19" t="s">
+        <v>158</v>
+      </c>
+      <c r="G19">
+        <v>1.77272727272727</v>
+      </c>
+      <c r="H19">
+        <v>321589.74808234</v>
+      </c>
+      <c r="I19">
+        <v>0.804064811607477</v>
+      </c>
+      <c r="J19">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.060563836339967</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>127</v>
+      </c>
+      <c r="C20">
+        <v>1.5719825141063899</v>
+      </c>
+      <c r="D20">
+        <v>355.37421751002699</v>
+      </c>
+      <c r="E20">
+        <v>420.395814642088</v>
+      </c>
+      <c r="F20" t="s">
+        <v>159</v>
+      </c>
+      <c r="G20">
+        <v>1.81636363636363</v>
+      </c>
+      <c r="H20">
+        <v>286741.00957474503</v>
+      </c>
+      <c r="I20">
+        <v>0.87850716168591203</v>
+      </c>
+      <c r="J20">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>0.84533243465466379</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D21">
+        <v>328.822071605914</v>
+      </c>
+      <c r="E21">
+        <v>318.08754981670802</v>
+      </c>
+      <c r="F21" t="s">
+        <v>160</v>
+      </c>
+      <c r="G21">
+        <v>1.78727272727272</v>
+      </c>
+      <c r="H21">
+        <v>318139.86709852598</v>
+      </c>
+      <c r="I21">
+        <v>0.83034940506079102</v>
+      </c>
+      <c r="J21">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0337470667914905</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>129</v>
+      </c>
+      <c r="C22">
+        <v>1.5727422431122799</v>
+      </c>
+      <c r="D22">
+        <v>946.03028739470801</v>
+      </c>
+      <c r="E22">
+        <v>935.00892045436603</v>
+      </c>
+      <c r="F22" t="s">
+        <v>161</v>
+      </c>
+      <c r="G22">
+        <v>1.82</v>
+      </c>
+      <c r="H22">
+        <v>314746.85255571501</v>
+      </c>
+      <c r="I22">
+        <v>1.82</v>
+      </c>
+      <c r="J22">
+        <f>Tabla2[[#This Row],[mismatch_w]]/Tabla2[[#This Row],[distance_w]]</f>
+        <v>1.0117874457657432</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F28" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82E474F6-C836-4628-9E19-F00913CCCF42}">
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="27.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="7" max="7" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D2">
+        <v>200.24192977416399</v>
+      </c>
+      <c r="E2">
+        <v>409.16815144556</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D3">
+        <v>297.26433233081701</v>
+      </c>
+      <c r="E3">
+        <v>608.20103868161004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D4">
+        <v>465.34719864343498</v>
+      </c>
+      <c r="E4">
+        <v>922.29689277279294</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D5">
+        <v>340.42059406021201</v>
+      </c>
+      <c r="E5">
+        <v>674.63145061642695</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C6">
+        <v>2.5335115471740099</v>
+      </c>
+      <c r="D6">
+        <v>105.441344951803</v>
+      </c>
+      <c r="E6">
+        <v>205.86913061351001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C7">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D7">
+        <v>349.43264790342198</v>
+      </c>
+      <c r="E7">
+        <v>713.07166755478204</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C8">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D8">
+        <v>285.606178623826</v>
+      </c>
+      <c r="E8">
+        <v>571.98514261387697</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C9">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D9">
+        <v>370.96257703029403</v>
+      </c>
+      <c r="E9">
+        <v>739.63753816609801</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C10">
+        <v>2.53293869747039</v>
+      </c>
+      <c r="D10">
+        <v>128.78253434620501</v>
+      </c>
+      <c r="E10">
+        <v>232.02676567453</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>139</v>
+      </c>
+      <c r="C11">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D11">
+        <v>491.43446599669397</v>
+      </c>
+      <c r="E11">
+        <v>974.80762374015205</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12">
+        <v>2.5334879904918801</v>
+      </c>
+      <c r="D12">
+        <v>49.503442635248803</v>
+      </c>
+      <c r="E12">
+        <v>95.0075841861605</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>141</v>
+      </c>
+      <c r="C13">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D13">
+        <v>82.504445103672694</v>
+      </c>
+      <c r="E13">
+        <v>163.82961508152599</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>142</v>
+      </c>
+      <c r="C14">
+        <v>2.53258718665366</v>
+      </c>
+      <c r="D14">
+        <v>78.210455735429505</v>
+      </c>
+      <c r="E14">
+        <v>129.85274641201599</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>143</v>
+      </c>
+      <c r="C15">
+        <v>2.5089117498814102</v>
+      </c>
+      <c r="D15">
+        <v>503.965081450208</v>
+      </c>
+      <c r="E15">
+        <v>1.8344893848013499</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>144</v>
+      </c>
+      <c r="C16">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D16">
+        <v>103.78141809812099</v>
+      </c>
+      <c r="E16">
+        <v>208.805960754457</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C17">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D17">
+        <v>268.27358903175298</v>
+      </c>
+      <c r="E17">
+        <v>541.122152277331</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>146</v>
+      </c>
+      <c r="C18">
+        <v>2.5191942701872501</v>
+      </c>
+      <c r="D18">
+        <v>758.63961987114396</v>
+      </c>
+      <c r="E18">
+        <v>419.92159188468901</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>147</v>
+      </c>
+      <c r="C19">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D19">
+        <v>118.869765959123</v>
+      </c>
+      <c r="E19">
+        <v>236.411309777003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>148</v>
+      </c>
+      <c r="C20">
+        <v>2.5335152099588698</v>
+      </c>
+      <c r="D20">
+        <v>27.825233125429801</v>
+      </c>
+      <c r="E20">
+        <v>56.084757389501199</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>149</v>
+      </c>
+      <c r="C21">
+        <v>2.5191942701872501</v>
+      </c>
+      <c r="D21">
+        <v>223.584843717398</v>
+      </c>
+      <c r="E21">
+        <v>141.15032931389999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD8DD79-C21B-42FF-8DFE-3955CE9BC814}">
   <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -770,30 +2330,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="C2" s="3">
-        <v>1.75514737917865</v>
+        <v>1.72143931068544</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="F2">
-        <v>1.841</v>
+        <v>1.8149999999999999</v>
       </c>
       <c r="G2" s="2">
-        <v>334628.96999999997</v>
+        <v>392269.99</v>
       </c>
       <c r="H2">
-        <v>0.86810699999999996</v>
+        <v>0.851159</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -822,111 +2382,111 @@
         <v>0.92507099999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="C4" s="3">
-        <v>1.75513882212879</v>
+        <v>1.75309618753157</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F4">
-        <v>1.91</v>
+        <v>1.845</v>
       </c>
       <c r="G4" s="2">
-        <v>338152.3</v>
+        <v>361994.7</v>
       </c>
       <c r="H4">
-        <v>0.91342599999999996</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.89156100000000005</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C5" s="3">
-        <v>1.75511970406575</v>
+        <v>1.74533799958452</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F5">
-        <v>1.859</v>
+        <v>1.8460000000000001</v>
       </c>
       <c r="G5" s="2">
-        <v>343097.64</v>
+        <v>414504.03</v>
       </c>
       <c r="H5">
-        <v>0.78561300000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.93656099999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C6" s="3">
-        <v>1.75509502690902</v>
+        <v>1.7537984301904901</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="F6">
-        <v>1.905</v>
+        <v>1.8480000000000001</v>
       </c>
       <c r="G6" s="2">
-        <v>333699.57</v>
+        <v>322689.89</v>
       </c>
       <c r="H6">
-        <v>0.89082899999999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.86023499999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="C7" s="3">
-        <v>1.7550735867325999</v>
+        <v>1.7512080548617801</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="F7">
-        <v>1.883</v>
+        <v>1.851</v>
       </c>
       <c r="G7" s="2">
-        <v>353694.83</v>
+        <v>317253.45</v>
       </c>
       <c r="H7">
-        <v>0.91786699999999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.87064699999999995</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>16</v>
       </c>
@@ -954,343 +2514,343 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C9" s="3">
-        <v>1.7547795458528499</v>
+        <v>1.7550735867325999</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F9">
-        <v>1.885</v>
+        <v>1.883</v>
       </c>
       <c r="G9" s="2">
-        <v>342950.36</v>
+        <v>353694.83</v>
       </c>
       <c r="H9">
-        <v>0.89133099999999998</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.91786699999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C10" s="3">
-        <v>1.7546794896511799</v>
+        <v>1.7117185958801899</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F10">
-        <v>1.875</v>
+        <v>1.8660000000000001</v>
       </c>
       <c r="G10" s="2">
-        <v>363907.11</v>
+        <v>291938.31</v>
       </c>
       <c r="H10">
-        <v>0.91680799999999996</v>
+        <v>0.91696200000000005</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1.75513882212879</v>
+      </c>
+      <c r="D11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11">
+        <v>1.91</v>
+      </c>
+      <c r="G11" s="2">
+        <v>338152.3</v>
+      </c>
+      <c r="H11">
+        <v>0.91342599999999996</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="3">
+        <v>1.7546794896511799</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12">
+        <v>1.875</v>
+      </c>
+      <c r="G12" s="2">
+        <v>363907.11</v>
+      </c>
+      <c r="H12">
+        <v>0.91680799999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="3">
+        <v>1.7543637471776099</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13">
+        <v>1.8759999999999999</v>
+      </c>
+      <c r="G13" s="2">
+        <v>348499.73</v>
+      </c>
+      <c r="H13">
+        <v>0.88633399999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>2</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B14" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C14" s="3">
         <v>1.7544618705931601</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D14" t="s">
         <v>6</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E14" t="s">
         <v>50</v>
       </c>
-      <c r="F11">
+      <c r="F14">
         <v>1.879</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G14" s="2">
         <v>342973.97</v>
       </c>
-      <c r="H11">
+      <c r="H14">
         <v>0.93385300000000004</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="3">
-        <v>1.7543637471776099</v>
-      </c>
-      <c r="D12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12">
-        <v>1.8759999999999999</v>
-      </c>
-      <c r="G12" s="2">
-        <v>348499.73</v>
-      </c>
-      <c r="H12">
-        <v>0.88633399999999996</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>7</v>
-      </c>
-      <c r="B13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="3">
-        <v>1.7541532442557299</v>
-      </c>
-      <c r="D13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13">
-        <v>1.897</v>
-      </c>
-      <c r="G13" s="2">
-        <v>353908.64</v>
-      </c>
-      <c r="H13">
-        <v>0.92070700000000005</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>21</v>
-      </c>
-      <c r="B14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="3">
-        <v>1.7537984301904901</v>
-      </c>
-      <c r="D14" t="s">
-        <v>47</v>
-      </c>
-      <c r="E14" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14">
-        <v>1.8480000000000001</v>
-      </c>
-      <c r="G14" s="2">
-        <v>322689.89</v>
-      </c>
-      <c r="H14">
-        <v>0.86023499999999997</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="3">
+        <v>1.75509502690902</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F15">
+        <v>1.905</v>
+      </c>
+      <c r="G15" s="2">
+        <v>333699.57</v>
+      </c>
+      <c r="H15">
+        <v>0.89082899999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="3">
+        <v>1.7547795458528499</v>
+      </c>
+      <c r="D16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16">
+        <v>1.885</v>
+      </c>
+      <c r="G16" s="2">
+        <v>342950.36</v>
+      </c>
+      <c r="H16">
+        <v>0.89133099999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>11</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B17" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C17" s="3">
         <v>1.75359996924416</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D17" t="s">
         <v>24</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E17" t="s">
         <v>60</v>
       </c>
-      <c r="F15">
+      <c r="F17">
         <v>1.887</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G17" s="2">
         <v>351491.95</v>
       </c>
-      <c r="H15">
+      <c r="H17">
         <v>0.90291600000000005</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>20</v>
-      </c>
-      <c r="B16" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="3">
-        <v>1.75309618753157</v>
-      </c>
-      <c r="D16" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" t="s">
-        <v>69</v>
-      </c>
-      <c r="F16">
-        <v>1.845</v>
-      </c>
-      <c r="G16" s="2">
-        <v>361994.7</v>
-      </c>
-      <c r="H16">
-        <v>0.89156100000000005</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>19</v>
-      </c>
-      <c r="B17" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" s="3">
-        <v>1.7512080548617801</v>
-      </c>
-      <c r="D17" t="s">
-        <v>40</v>
-      </c>
-      <c r="E17" t="s">
-        <v>68</v>
-      </c>
-      <c r="F17">
-        <v>1.851</v>
-      </c>
-      <c r="G17" s="2">
-        <v>317253.45</v>
-      </c>
-      <c r="H17">
-        <v>0.87064699999999995</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C18" s="3">
-        <v>1.74533799958452</v>
+        <v>1.7541532442557299</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="E18" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="F18">
-        <v>1.8460000000000001</v>
+        <v>1.897</v>
       </c>
       <c r="G18" s="2">
-        <v>414504.03</v>
+        <v>353908.64</v>
       </c>
       <c r="H18">
-        <v>0.93656099999999998</v>
+        <v>0.92070700000000005</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="C19" s="3">
-        <v>1.7217416663736</v>
+        <v>1.75514737917865</v>
       </c>
       <c r="D19" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="E19" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="F19">
-        <v>1.9319999999999999</v>
+        <v>1.841</v>
       </c>
       <c r="G19" s="2">
-        <v>309284.96999999997</v>
+        <v>334628.96999999997</v>
       </c>
       <c r="H19">
-        <v>0.86438000000000004</v>
+        <v>0.86810699999999996</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C20" s="3">
-        <v>1.72143931068544</v>
+        <v>1.75511970406575</v>
       </c>
       <c r="D20" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E20" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F20">
-        <v>1.8149999999999999</v>
+        <v>1.859</v>
       </c>
       <c r="G20" s="2">
-        <v>392269.99</v>
+        <v>343097.64</v>
       </c>
       <c r="H20">
-        <v>0.851159</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.78561300000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C21" s="3">
-        <v>1.7117185958801899</v>
+        <v>1.7217416663736</v>
       </c>
       <c r="D21" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F21">
-        <v>1.8660000000000001</v>
+        <v>1.9319999999999999</v>
       </c>
       <c r="G21" s="2">
-        <v>291938.31</v>
+        <v>309284.96999999997</v>
       </c>
       <c r="H21">
-        <v>0.91696200000000005</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.86438000000000004</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1</v>
       </c>
@@ -1348,7 +2908,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD728884-C592-489A-A034-49A00860CA4C}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1390,7 +2950,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{405D8D96-F676-4056-8F48-CADB3D12E67E}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>